<commit_message>
patch: Implementei “PÁGINA OFICIAL” abaixo do nome, com sublinhado ao passar o cursor, e suporte à coluna no editor. A atualização do site ficou bloqueada por uma inconsistência na planilha: “Direção” foi renomeada para “Centro Multidisciplinar de Angicos”, mas os servidores ainda usam “Direção”; o campo “Endereço” também contém espaços. Posso uniformizar o setor como “Centro Multidisciplinar de Angicos” e usar centro-multidisciplinar-de-angicos no endereço?
</commit_message>
<xml_diff>
--- a/Corpo Administrativo.xlsx
+++ b/Corpo Administrativo.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\leanm\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B991B24A-625B-468C-AAF2-E077788193FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{174FE314-3C62-4786-A02D-268E4187AEE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TAES" sheetId="4" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="590" uniqueCount="336">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="596" uniqueCount="342">
   <si>
     <t>Siape</t>
   </si>
@@ -862,9 +862,6 @@
     <t>#f4effc</t>
   </si>
   <si>
-    <t>direcao</t>
-  </si>
-  <si>
     <t>#22677b</t>
   </si>
   <si>
@@ -1034,16 +1031,37 @@
   </si>
   <si>
     <t>DOUTORADO</t>
+  </si>
+  <si>
+    <t>Página</t>
+  </si>
+  <si>
+    <t>https://coaeangicos.ufersa.edu.br/</t>
+  </si>
+  <si>
+    <t>https://angicos.ufersa.edu.br/campus-coord-academica-sobre-a-caang/</t>
+  </si>
+  <si>
+    <t>https://angicos.ufersa.edu.br/coordenacao-de-planejamento-e-administracao/</t>
+  </si>
+  <si>
+    <t>https://angicos.ufersa.edu.br/biblioteca/</t>
+  </si>
+  <si>
+    <t>https://angicos.ufersa.edu.br/secretaria-cma/</t>
+  </si>
+  <si>
+    <t>Centro Multidisciplinar de Angicos</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="d/m/yyyy"/>
   </numFmts>
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -1092,6 +1110,12 @@
       <sz val="12"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="10"/>
+      <color theme="10"/>
+      <name val="Arial"/>
     </font>
   </fonts>
   <fills count="6">
@@ -1159,10 +1183,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -1197,22 +1222,23 @@
     <xf numFmtId="0" fontId="8" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="49" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="49" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="49" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="49" fontId="2" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hiperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
-    <ext uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
     </ext>
-    <ext uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
       <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
@@ -1413,7 +1439,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AC1000"/>
   <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1445,7 +1471,7 @@
         <v>3</v>
       </c>
       <c r="E1" s="22" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="F1" s="16" t="s">
         <v>4</v>
@@ -1500,7 +1526,7 @@
         <v>46</v>
       </c>
       <c r="E2" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="F2" s="4" t="s">
         <v>47</v>
@@ -1508,10 +1534,8 @@
       <c r="G2" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="H2" s="23" t="inlineStr">
-        <is>
-          <t>30-12</t>
-        </is>
+      <c r="H2" s="12">
+        <v>35063</v>
       </c>
       <c r="I2" s="5" t="s">
         <v>15</v>
@@ -1557,7 +1581,7 @@
         <v>12</v>
       </c>
       <c r="E3" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="F3" s="4" t="s">
         <v>13</v>
@@ -1565,10 +1589,8 @@
       <c r="G3" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="H3" s="24" t="inlineStr">
-        <is>
-          <t>27-01</t>
-        </is>
+      <c r="H3" s="4">
+        <v>33996</v>
       </c>
       <c r="I3" s="5" t="s">
         <v>15</v>
@@ -1614,7 +1636,7 @@
         <v>52</v>
       </c>
       <c r="E4" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="F4" s="8" t="s">
         <v>47</v>
@@ -1622,10 +1644,8 @@
       <c r="G4" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="H4" s="25" t="inlineStr">
-        <is>
-          <t>17-06</t>
-        </is>
+      <c r="H4" s="8">
+        <v>28293</v>
       </c>
       <c r="I4" s="10" t="s">
         <v>15</v>
@@ -1671,7 +1691,7 @@
         <v>89</v>
       </c>
       <c r="E5" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="F5" s="8" t="s">
         <v>90</v>
@@ -1679,10 +1699,8 @@
       <c r="G5" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="H5" s="25" t="inlineStr">
-        <is>
-          <t>09-10</t>
-        </is>
+      <c r="H5" s="8">
+        <v>31329</v>
       </c>
       <c r="I5" s="10" t="s">
         <v>15</v>
@@ -1728,7 +1746,7 @@
         <v>93</v>
       </c>
       <c r="E6" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="F6" s="4" t="s">
         <v>90</v>
@@ -1736,10 +1754,8 @@
       <c r="G6" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="H6" s="23" t="inlineStr">
-        <is>
-          <t>14-11</t>
-        </is>
+      <c r="H6" s="12">
+        <v>33191</v>
       </c>
       <c r="I6" s="5" t="s">
         <v>15</v>
@@ -1785,7 +1801,7 @@
         <v>106</v>
       </c>
       <c r="E7" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="F7" s="1" t="s">
         <v>107</v>
@@ -1793,10 +1809,8 @@
       <c r="G7" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="H7" s="24" t="inlineStr">
-        <is>
-          <t>10-09</t>
-        </is>
+      <c r="H7" s="4">
+        <v>27647</v>
       </c>
       <c r="I7" s="5" t="s">
         <v>15</v>
@@ -1842,7 +1856,7 @@
         <v>19</v>
       </c>
       <c r="E8" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="F8" s="8" t="s">
         <v>13</v>
@@ -1850,10 +1864,8 @@
       <c r="G8" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="H8" s="25" t="inlineStr">
-        <is>
-          <t>19-06</t>
-        </is>
+      <c r="H8" s="8">
+        <v>31947</v>
       </c>
       <c r="I8" s="10" t="s">
         <v>15</v>
@@ -1899,7 +1911,7 @@
         <v>111</v>
       </c>
       <c r="E9" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="F9" s="9" t="s">
         <v>107</v>
@@ -1907,10 +1919,8 @@
       <c r="G9" s="9" t="s">
         <v>112</v>
       </c>
-      <c r="H9" s="25" t="inlineStr">
-        <is>
-          <t>01-03</t>
-        </is>
+      <c r="H9" s="8">
+        <v>23437</v>
       </c>
       <c r="I9" s="10" t="s">
         <v>15</v>
@@ -1954,7 +1964,7 @@
         <v>115</v>
       </c>
       <c r="E10" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="F10" s="1" t="s">
         <v>107</v>
@@ -1962,10 +1972,8 @@
       <c r="G10" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="H10" s="24" t="inlineStr">
-        <is>
-          <t>06-07</t>
-        </is>
+      <c r="H10" s="4">
+        <v>30869</v>
       </c>
       <c r="I10" s="5" t="s">
         <v>15</v>
@@ -2011,7 +2019,7 @@
         <v>119</v>
       </c>
       <c r="E11" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="F11" s="9" t="s">
         <v>107</v>
@@ -2019,10 +2027,8 @@
       <c r="G11" s="9" t="s">
         <v>108</v>
       </c>
-      <c r="H11" s="25" t="inlineStr">
-        <is>
-          <t>24-06</t>
-        </is>
+      <c r="H11" s="8">
+        <v>32318</v>
       </c>
       <c r="I11" s="10" t="s">
         <v>15</v>
@@ -2068,7 +2074,7 @@
         <v>96</v>
       </c>
       <c r="E12" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="F12" s="8" t="s">
         <v>90</v>
@@ -2076,10 +2082,8 @@
       <c r="G12" s="9" t="s">
         <v>97</v>
       </c>
-      <c r="H12" s="26" t="inlineStr">
-        <is>
-          <t>23-12</t>
-        </is>
+      <c r="H12" s="13">
+        <v>32134</v>
       </c>
       <c r="I12" s="10" t="s">
         <v>15</v>
@@ -2125,7 +2129,7 @@
         <v>56</v>
       </c>
       <c r="E13" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="F13" s="4" t="s">
         <v>47</v>
@@ -2133,10 +2137,8 @@
       <c r="G13" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="H13" s="24" t="inlineStr">
-        <is>
-          <t>14-01</t>
-        </is>
+      <c r="H13" s="4">
+        <v>31061</v>
       </c>
       <c r="I13" s="5" t="s">
         <v>15</v>
@@ -2182,7 +2184,7 @@
         <v>59</v>
       </c>
       <c r="E14" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="F14" s="8" t="s">
         <v>47</v>
@@ -2190,10 +2192,8 @@
       <c r="G14" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="H14" s="25" t="inlineStr">
-        <is>
-          <t>24-01</t>
-        </is>
+      <c r="H14" s="8">
+        <v>33262</v>
       </c>
       <c r="I14" s="10" t="s">
         <v>15</v>
@@ -2239,7 +2239,7 @@
         <v>152</v>
       </c>
       <c r="E15" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="F15" s="1" t="s">
         <v>153</v>
@@ -2247,10 +2247,8 @@
       <c r="G15" s="1" t="s">
         <v>154</v>
       </c>
-      <c r="H15" s="23" t="inlineStr">
-        <is>
-          <t>29-12</t>
-        </is>
+      <c r="H15" s="12">
+        <v>33601</v>
       </c>
       <c r="I15" s="5" t="s">
         <v>15</v>
@@ -2296,7 +2294,7 @@
         <v>165</v>
       </c>
       <c r="E16" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="F16" s="9" t="s">
         <v>153</v>
@@ -2304,10 +2302,8 @@
       <c r="G16" s="9" t="s">
         <v>166</v>
       </c>
-      <c r="H16" s="25" t="inlineStr">
-        <is>
-          <t>27-05</t>
-        </is>
+      <c r="H16" s="8">
+        <v>27907</v>
       </c>
       <c r="I16" s="10" t="s">
         <v>15</v>
@@ -2353,7 +2349,7 @@
         <v>169</v>
       </c>
       <c r="E17" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="F17" s="1" t="s">
         <v>153</v>
@@ -2361,10 +2357,8 @@
       <c r="G17" s="1" t="s">
         <v>170</v>
       </c>
-      <c r="H17" s="24" t="inlineStr">
-        <is>
-          <t>02-12</t>
-        </is>
+      <c r="H17" s="4">
+        <v>33940</v>
       </c>
       <c r="I17" s="5" t="s">
         <v>15</v>
@@ -2410,7 +2404,7 @@
         <v>22</v>
       </c>
       <c r="E18" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="F18" s="4" t="s">
         <v>13</v>
@@ -2418,10 +2412,8 @@
       <c r="G18" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="H18" s="24" t="inlineStr">
-        <is>
-          <t>14-01</t>
-        </is>
+      <c r="H18" s="4">
+        <v>31426</v>
       </c>
       <c r="I18" s="5" t="s">
         <v>15</v>
@@ -2467,7 +2459,7 @@
         <v>122</v>
       </c>
       <c r="E19" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="F19" s="1" t="s">
         <v>107</v>
@@ -2475,10 +2467,8 @@
       <c r="G19" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="H19" s="24" t="inlineStr">
-        <is>
-          <t>23-05</t>
-        </is>
+      <c r="H19" s="4">
+        <v>32286</v>
       </c>
       <c r="I19" s="5" t="s">
         <v>15</v>
@@ -2524,7 +2514,7 @@
         <v>26</v>
       </c>
       <c r="E20" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="F20" s="8" t="s">
         <v>13</v>
@@ -2532,10 +2522,8 @@
       <c r="G20" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="H20" s="25" t="inlineStr">
-        <is>
-          <t>25-01</t>
-        </is>
+      <c r="H20" s="8">
+        <v>31072</v>
       </c>
       <c r="I20" s="10" t="s">
         <v>15</v>
@@ -2581,7 +2569,7 @@
         <v>126</v>
       </c>
       <c r="E21" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="F21" s="9" t="s">
         <v>107</v>
@@ -2589,10 +2577,8 @@
       <c r="G21" s="9" t="s">
         <v>127</v>
       </c>
-      <c r="H21" s="25" t="inlineStr">
-        <is>
-          <t>27-09</t>
-        </is>
+      <c r="H21" s="8">
+        <v>36065</v>
       </c>
       <c r="I21" s="10" t="s">
         <v>15</v>
@@ -2638,7 +2624,7 @@
         <v>64</v>
       </c>
       <c r="E22" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="F22" s="4" t="s">
         <v>47</v>
@@ -2646,10 +2632,8 @@
       <c r="G22" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="H22" s="23" t="inlineStr">
-        <is>
-          <t>10-11</t>
-        </is>
+      <c r="H22" s="12">
+        <v>32457</v>
       </c>
       <c r="I22" s="5" t="s">
         <v>15</v>
@@ -2695,7 +2679,7 @@
         <v>31</v>
       </c>
       <c r="E23" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="F23" s="4" t="s">
         <v>13</v>
@@ -2703,10 +2687,8 @@
       <c r="G23" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="H23" s="23" t="inlineStr">
-        <is>
-          <t>20-12</t>
-        </is>
+      <c r="H23" s="12">
+        <v>32497</v>
       </c>
       <c r="I23" s="5" t="s">
         <v>15</v>
@@ -2752,7 +2734,7 @@
         <v>130</v>
       </c>
       <c r="E24" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="F24" s="1" t="s">
         <v>107</v>
@@ -2760,10 +2742,8 @@
       <c r="G24" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="H24" s="24" t="inlineStr">
-        <is>
-          <t>18-08</t>
-        </is>
+      <c r="H24" s="4">
+        <v>31642</v>
       </c>
       <c r="I24" s="5" t="s">
         <v>15</v>
@@ -2809,7 +2789,7 @@
         <v>67</v>
       </c>
       <c r="E25" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="F25" s="8" t="s">
         <v>47</v>
@@ -2817,10 +2797,8 @@
       <c r="G25" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="H25" s="25" t="inlineStr">
-        <is>
-          <t>04-08</t>
-        </is>
+      <c r="H25" s="8">
+        <v>31628</v>
       </c>
       <c r="I25" s="10" t="s">
         <v>15</v>
@@ -2866,7 +2844,7 @@
         <v>157</v>
       </c>
       <c r="E26" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="F26" s="9" t="s">
         <v>153</v>
@@ -2874,10 +2852,8 @@
       <c r="G26" s="9" t="s">
         <v>154</v>
       </c>
-      <c r="H26" s="25" t="inlineStr">
-        <is>
-          <t>10-04</t>
-        </is>
+      <c r="H26" s="8">
+        <v>31147</v>
       </c>
       <c r="I26" s="10" t="s">
         <v>15</v>
@@ -2923,7 +2899,7 @@
         <v>173</v>
       </c>
       <c r="E27" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="F27" s="9" t="s">
         <v>153</v>
@@ -2931,10 +2907,8 @@
       <c r="G27" s="9" t="s">
         <v>174</v>
       </c>
-      <c r="H27" s="25" t="inlineStr">
-        <is>
-          <t>20-09</t>
-        </is>
+      <c r="H27" s="8">
+        <v>29849</v>
       </c>
       <c r="I27" s="10" t="s">
         <v>15</v>
@@ -2980,7 +2954,7 @@
         <v>35</v>
       </c>
       <c r="E28" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="F28" s="8" t="s">
         <v>13</v>
@@ -2988,10 +2962,8 @@
       <c r="G28" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="H28" s="25" t="inlineStr">
-        <is>
-          <t>29-05</t>
-        </is>
+      <c r="H28" s="8">
+        <v>33022</v>
       </c>
       <c r="I28" s="10" t="s">
         <v>15</v>
@@ -3037,7 +3009,7 @@
         <v>71</v>
       </c>
       <c r="E29" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="F29" s="4" t="s">
         <v>47</v>
@@ -3045,10 +3017,8 @@
       <c r="G29" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="H29" s="24" t="inlineStr">
-        <is>
-          <t>03-05</t>
-        </is>
+      <c r="H29" s="4">
+        <v>30439</v>
       </c>
       <c r="I29" s="5" t="s">
         <v>15</v>
@@ -3094,7 +3064,7 @@
         <v>134</v>
       </c>
       <c r="E30" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="F30" s="9" t="s">
         <v>107</v>
@@ -3102,10 +3072,8 @@
       <c r="G30" s="9" t="s">
         <v>97</v>
       </c>
-      <c r="H30" s="25" t="inlineStr">
-        <is>
-          <t>23-05</t>
-        </is>
+      <c r="H30" s="8">
+        <v>27537</v>
       </c>
       <c r="I30" s="10" t="s">
         <v>15</v>
@@ -3151,7 +3119,7 @@
         <v>100</v>
       </c>
       <c r="E31" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="F31" s="4" t="s">
         <v>90</v>
@@ -3159,10 +3127,8 @@
       <c r="G31" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="H31" s="23" t="inlineStr">
-        <is>
-          <t>20-10</t>
-        </is>
+      <c r="H31" s="12">
+        <v>33897</v>
       </c>
       <c r="I31" s="5" t="s">
         <v>15</v>
@@ -3208,7 +3174,7 @@
         <v>75</v>
       </c>
       <c r="E32" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="F32" s="8" t="s">
         <v>47</v>
@@ -3216,10 +3182,8 @@
       <c r="G32" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="H32" s="25" t="inlineStr">
-        <is>
-          <t>30-08</t>
-        </is>
+      <c r="H32" s="8">
+        <v>29097</v>
       </c>
       <c r="I32" s="10" t="s">
         <v>15</v>
@@ -3265,7 +3229,7 @@
         <v>78</v>
       </c>
       <c r="E33" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="F33" s="4" t="s">
         <v>47</v>
@@ -3273,10 +3237,8 @@
       <c r="G33" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="H33" s="23" t="inlineStr">
-        <is>
-          <t>21-10</t>
-        </is>
+      <c r="H33" s="12">
+        <v>22940</v>
       </c>
       <c r="I33" s="5" t="s">
         <v>15</v>
@@ -3322,7 +3284,7 @@
         <v>38</v>
       </c>
       <c r="E34" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="F34" s="4" t="s">
         <v>13</v>
@@ -3330,10 +3292,8 @@
       <c r="G34" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="H34" s="24" t="inlineStr">
-        <is>
-          <t>05-10</t>
-        </is>
+      <c r="H34" s="4">
+        <v>31325</v>
       </c>
       <c r="I34" s="5" t="s">
         <v>15</v>
@@ -3379,7 +3339,7 @@
         <v>137</v>
       </c>
       <c r="E35" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="F35" s="1" t="s">
         <v>107</v>
@@ -3387,10 +3347,8 @@
       <c r="G35" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="H35" s="24" t="inlineStr">
-        <is>
-          <t>02-07</t>
-        </is>
+      <c r="H35" s="4">
+        <v>24655</v>
       </c>
       <c r="I35" s="5" t="s">
         <v>15</v>
@@ -3436,7 +3394,7 @@
         <v>42</v>
       </c>
       <c r="E36" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="F36" s="8" t="s">
         <v>13</v>
@@ -3444,10 +3402,8 @@
       <c r="G36" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="H36" s="26" t="inlineStr">
-        <is>
-          <t>30-10</t>
-        </is>
+      <c r="H36" s="13">
+        <v>37194</v>
       </c>
       <c r="I36" s="10" t="s">
         <v>15</v>
@@ -3493,7 +3449,7 @@
         <v>161</v>
       </c>
       <c r="E37" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="F37" s="1" t="s">
         <v>153</v>
@@ -3501,10 +3457,8 @@
       <c r="G37" s="1" t="s">
         <v>154</v>
       </c>
-      <c r="H37" s="24" t="inlineStr">
-        <is>
-          <t>03-08</t>
-        </is>
+      <c r="H37" s="4">
+        <v>29801</v>
       </c>
       <c r="I37" s="5" t="s">
         <v>15</v>
@@ -3550,7 +3504,7 @@
         <v>81</v>
       </c>
       <c r="E38" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="F38" s="8" t="s">
         <v>47</v>
@@ -3558,10 +3512,8 @@
       <c r="G38" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="H38" s="26" t="inlineStr">
-        <is>
-          <t>10-10</t>
-        </is>
+      <c r="H38" s="13">
+        <v>25486</v>
       </c>
       <c r="I38" s="10" t="s">
         <v>15</v>
@@ -3607,7 +3559,7 @@
         <v>141</v>
       </c>
       <c r="E39" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="F39" s="9" t="s">
         <v>107</v>
@@ -3615,10 +3567,8 @@
       <c r="G39" s="9" t="s">
         <v>138</v>
       </c>
-      <c r="H39" s="25" t="inlineStr">
-        <is>
-          <t>07-02</t>
-        </is>
+      <c r="H39" s="8">
+        <v>31450</v>
       </c>
       <c r="I39" s="10" t="s">
         <v>15</v>
@@ -3664,7 +3614,7 @@
         <v>144</v>
       </c>
       <c r="E40" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="F40" s="1" t="s">
         <v>107</v>
@@ -3672,10 +3622,8 @@
       <c r="G40" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="H40" s="24" t="inlineStr">
-        <is>
-          <t>12-04</t>
-        </is>
+      <c r="H40" s="4">
+        <v>28957</v>
       </c>
       <c r="I40" s="5" t="s">
         <v>15</v>
@@ -3684,7 +3632,7 @@
         <v>15</v>
       </c>
       <c r="K40" s="1" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="L40" s="6" t="s">
         <v>244</v>
@@ -3721,7 +3669,7 @@
         <v>148</v>
       </c>
       <c r="E41" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="F41" s="9" t="s">
         <v>107</v>
@@ -3729,10 +3677,8 @@
       <c r="G41" s="9" t="s">
         <v>127</v>
       </c>
-      <c r="H41" s="25" t="inlineStr">
-        <is>
-          <t>14-06</t>
-        </is>
+      <c r="H41" s="8">
+        <v>37421</v>
       </c>
       <c r="I41" s="10" t="s">
         <v>15</v>
@@ -3778,7 +3724,7 @@
         <v>103</v>
       </c>
       <c r="E42" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="F42" s="8" t="s">
         <v>90</v>
@@ -3786,10 +3732,8 @@
       <c r="G42" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="H42" s="25" t="inlineStr">
-        <is>
-          <t>01-09</t>
-        </is>
+      <c r="H42" s="8">
+        <v>31656</v>
       </c>
       <c r="I42" s="10" t="s">
         <v>15</v>
@@ -3835,7 +3779,7 @@
         <v>85</v>
       </c>
       <c r="E43" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="F43" s="4" t="s">
         <v>47</v>
@@ -3843,10 +3787,8 @@
       <c r="G43" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="H43" s="24" t="inlineStr">
-        <is>
-          <t>21-09</t>
-        </is>
+      <c r="H43" s="4">
+        <v>30215</v>
       </c>
       <c r="I43" s="5" t="s">
         <v>15</v>
@@ -33547,7 +33489,7 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:AC1" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <sortState ref="A2:AC43">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:AC43">
       <sortCondition ref="B1"/>
     </sortState>
   </autoFilter>
@@ -33557,16 +33499,17 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="36" customWidth="1"/>
     <col min="2" max="2" width="60" customWidth="1"/>
     <col min="3" max="3" width="30" customWidth="1"/>
     <col min="4" max="5" width="16" customWidth="1"/>
+    <col min="6" max="6" width="33.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="19" t="s">
         <v>259</v>
       </c>
@@ -33582,8 +33525,11 @@
       <c r="E1" s="19" t="s">
         <v>262</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="F1" s="19" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="18" t="s">
         <v>263</v>
       </c>
@@ -33599,8 +33545,11 @@
       <c r="E2" s="18" t="s">
         <v>265</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="F2" s="24" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="18" t="s">
         <v>266</v>
       </c>
@@ -33616,8 +33565,11 @@
       <c r="E3" s="18" t="s">
         <v>269</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="F3" s="23" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="18" t="s">
         <v>270</v>
       </c>
@@ -33633,8 +33585,11 @@
       <c r="E4" s="18" t="s">
         <v>273</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="F4" s="23" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="18" t="s">
         <v>274</v>
       </c>
@@ -33650,25 +33605,41 @@
       <c r="E5" s="18" t="s">
         <v>277</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="F5" s="23" t="s">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="18" t="s">
+        <v>341</v>
+      </c>
+      <c r="B6" s="18" t="s">
+        <v>341</v>
+      </c>
+      <c r="C6" s="18" t="s">
+        <v>341</v>
+      </c>
+      <c r="D6" s="18" t="s">
         <v>278</v>
       </c>
-      <c r="B6" s="18" t="s">
-        <v>153</v>
-      </c>
-      <c r="C6" s="18" t="s">
-        <v>153</v>
-      </c>
-      <c r="D6" s="18" t="s">
+      <c r="E6" s="18" t="s">
         <v>279</v>
       </c>
-      <c r="E6" s="18" t="s">
-        <v>280</v>
-      </c>
+      <c r="F6" s="23" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="F7" s="24"/>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="F4" r:id="rId1" xr:uid="{DDD35E56-2970-4160-8348-2222639D6240}"/>
+    <hyperlink ref="F3" r:id="rId2" xr:uid="{8CEDDEAA-57AC-42FB-BFC2-36D17213FBD5}"/>
+    <hyperlink ref="F5" r:id="rId3" xr:uid="{0D117D76-BBED-470A-91C6-6511C49E8F1A}"/>
+    <hyperlink ref="F6" r:id="rId4" xr:uid="{C42B1848-5BB8-4387-8E3B-8869CE883310}"/>
+    <hyperlink ref="F2" r:id="rId5" xr:uid="{81E30D7E-F42C-42C7-8A99-E868C5F7D7F0}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -33696,7 +33667,7 @@
     </row>
     <row r="2" spans="1:3" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="18" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="B2" s="18" t="s">
         <v>13</v>
@@ -33707,7 +33678,7 @@
     </row>
     <row r="3" spans="1:3" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="18" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="B3" s="18" t="s">
         <v>13</v>
@@ -33718,7 +33689,7 @@
     </row>
     <row r="4" spans="1:3" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="18" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="B4" s="18" t="s">
         <v>47</v>
@@ -33729,7 +33700,7 @@
     </row>
     <row r="5" spans="1:3" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="18" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="B5" s="18" t="s">
         <v>47</v>
@@ -33740,7 +33711,7 @@
     </row>
     <row r="6" spans="1:3" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="18" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="B6" s="18" t="s">
         <v>47</v>
@@ -33751,7 +33722,7 @@
     </row>
     <row r="7" spans="1:3" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="18" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="B7" s="18" t="s">
         <v>90</v>
@@ -33762,7 +33733,7 @@
     </row>
     <row r="8" spans="1:3" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="18" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="B8" s="18" t="s">
         <v>90</v>
@@ -33773,7 +33744,7 @@
     </row>
     <row r="9" spans="1:3" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="18" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="B9" s="18" t="s">
         <v>107</v>
@@ -33784,7 +33755,7 @@
     </row>
     <row r="10" spans="1:3" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="18" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="B10" s="18" t="s">
         <v>107</v>
@@ -33795,7 +33766,7 @@
     </row>
     <row r="11" spans="1:3" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="18" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="B11" s="18" t="s">
         <v>107</v>
@@ -33806,7 +33777,7 @@
     </row>
     <row r="12" spans="1:3" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="18" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="B12" s="18" t="s">
         <v>107</v>
@@ -33817,7 +33788,7 @@
     </row>
     <row r="13" spans="1:3" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="18" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B13" s="18" t="s">
         <v>107</v>
@@ -33828,7 +33799,7 @@
     </row>
     <row r="14" spans="1:3" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="18" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="B14" s="18" t="s">
         <v>107</v>
@@ -33839,7 +33810,7 @@
     </row>
     <row r="15" spans="1:3" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="18" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="B15" s="18" t="s">
         <v>107</v>
@@ -33850,10 +33821,10 @@
     </row>
     <row r="16" spans="1:3" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="18" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="B16" s="18" t="s">
-        <v>153</v>
+        <v>341</v>
       </c>
       <c r="C16" s="18" t="s">
         <v>154</v>
@@ -33861,10 +33832,10 @@
     </row>
     <row r="17" spans="1:3" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="18" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="B17" s="18" t="s">
-        <v>153</v>
+        <v>341</v>
       </c>
       <c r="C17" s="18" t="s">
         <v>166</v>
@@ -33872,10 +33843,10 @@
     </row>
     <row r="18" spans="1:3" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="18" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="B18" s="18" t="s">
-        <v>153</v>
+        <v>341</v>
       </c>
       <c r="C18" s="18" t="s">
         <v>170</v>
@@ -33883,10 +33854,10 @@
     </row>
     <row r="19" spans="1:3" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="18" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="B19" s="18" t="s">
-        <v>153</v>
+        <v>341</v>
       </c>
       <c r="C19" s="18" t="s">
         <v>174</v>
@@ -33908,122 +33879,122 @@
   <sheetData>
     <row r="1" spans="1:2" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="21" t="s">
+        <v>298</v>
+      </c>
+      <c r="B1" s="21" t="s">
         <v>299</v>
-      </c>
-      <c r="B1" s="21" t="s">
-        <v>300</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="64.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="20" t="s">
+        <v>300</v>
+      </c>
+      <c r="B2" s="20" t="s">
         <v>301</v>
-      </c>
-      <c r="B2" s="20" t="s">
-        <v>302</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="64.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="20" t="s">
+        <v>302</v>
+      </c>
+      <c r="B3" s="20" t="s">
         <v>303</v>
-      </c>
-      <c r="B3" s="20" t="s">
-        <v>304</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="64.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="20" t="s">
+        <v>304</v>
+      </c>
+      <c r="B4" s="20" t="s">
         <v>305</v>
-      </c>
-      <c r="B4" s="20" t="s">
-        <v>306</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="64.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="20" t="s">
+        <v>306</v>
+      </c>
+      <c r="B5" s="20" t="s">
         <v>307</v>
-      </c>
-      <c r="B5" s="20" t="s">
-        <v>308</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="64.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="20" t="s">
+        <v>308</v>
+      </c>
+      <c r="B6" s="20" t="s">
         <v>309</v>
-      </c>
-      <c r="B6" s="20" t="s">
-        <v>310</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="64.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="20" t="s">
+        <v>310</v>
+      </c>
+      <c r="B7" s="20" t="s">
         <v>311</v>
-      </c>
-      <c r="B7" s="20" t="s">
-        <v>312</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="64.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="20" t="s">
+        <v>312</v>
+      </c>
+      <c r="B8" s="20" t="s">
         <v>313</v>
-      </c>
-      <c r="B8" s="20" t="s">
-        <v>314</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="64.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="20" t="s">
+        <v>314</v>
+      </c>
+      <c r="B9" s="20" t="s">
         <v>315</v>
-      </c>
-      <c r="B9" s="20" t="s">
-        <v>316</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="64.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="20" t="s">
+        <v>316</v>
+      </c>
+      <c r="B10" s="20" t="s">
         <v>317</v>
-      </c>
-      <c r="B10" s="20" t="s">
-        <v>318</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="64.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="20" t="s">
+        <v>318</v>
+      </c>
+      <c r="B11" s="20" t="s">
         <v>319</v>
-      </c>
-      <c r="B11" s="20" t="s">
-        <v>320</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="64.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="20" t="s">
+        <v>320</v>
+      </c>
+      <c r="B12" s="20" t="s">
         <v>321</v>
-      </c>
-      <c r="B12" s="20" t="s">
-        <v>322</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="64.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="20" t="s">
+        <v>322</v>
+      </c>
+      <c r="B13" s="20" t="s">
         <v>323</v>
-      </c>
-      <c r="B13" s="20" t="s">
-        <v>324</v>
       </c>
     </row>
     <row r="14" spans="1:2" ht="64.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="20" t="s">
+        <v>324</v>
+      </c>
+      <c r="B14" s="20" t="s">
         <v>325</v>
-      </c>
-      <c r="B14" s="20" t="s">
-        <v>326</v>
       </c>
     </row>
     <row r="15" spans="1:2" ht="64.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="20" t="s">
+        <v>326</v>
+      </c>
+      <c r="B15" s="20" t="s">
         <v>327</v>
-      </c>
-      <c r="B15" s="20" t="s">
-        <v>328</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
patch: Corrigido: - Padronizei o Centro Multidisciplinar de Angicos e seus seis servidores na planilha. - Gerei novamente as páginas com os cinco links PÁGINA OFICIAL, abaixo dos nomes, com sublinhado ao passar o cursor. - Validei os arquivos do deploy e os oito testes passaram. As alterações estão locais. Faça commit e push, incluindo a nova pasta centro-multidisciplinar-de-angicos, para atualizar o GitHub Pages.
</commit_message>
<xml_diff>
--- a/Corpo Administrativo.xlsx
+++ b/Corpo Administrativo.xlsx
@@ -2241,8 +2241,10 @@
       <c r="E15" t="s">
         <v>332</v>
       </c>
-      <c r="F15" s="1" t="s">
-        <v>153</v>
+      <c r="F15" s="1" t="inlineStr">
+        <is>
+          <t>Centro Multidisciplinar de Angicos</t>
+        </is>
       </c>
       <c r="G15" s="1" t="s">
         <v>154</v>
@@ -2296,8 +2298,10 @@
       <c r="E16" t="s">
         <v>330</v>
       </c>
-      <c r="F16" s="9" t="s">
-        <v>153</v>
+      <c r="F16" s="9" t="inlineStr">
+        <is>
+          <t>Centro Multidisciplinar de Angicos</t>
+        </is>
       </c>
       <c r="G16" s="9" t="s">
         <v>166</v>
@@ -2351,8 +2355,10 @@
       <c r="E17" t="s">
         <v>330</v>
       </c>
-      <c r="F17" s="1" t="s">
-        <v>153</v>
+      <c r="F17" s="1" t="inlineStr">
+        <is>
+          <t>Centro Multidisciplinar de Angicos</t>
+        </is>
       </c>
       <c r="G17" s="1" t="s">
         <v>170</v>
@@ -2846,8 +2852,10 @@
       <c r="E26" t="s">
         <v>332</v>
       </c>
-      <c r="F26" s="9" t="s">
-        <v>153</v>
+      <c r="F26" s="9" t="inlineStr">
+        <is>
+          <t>Centro Multidisciplinar de Angicos</t>
+        </is>
       </c>
       <c r="G26" s="9" t="s">
         <v>154</v>
@@ -2901,8 +2909,10 @@
       <c r="E27" t="s">
         <v>332</v>
       </c>
-      <c r="F27" s="9" t="s">
-        <v>153</v>
+      <c r="F27" s="9" t="inlineStr">
+        <is>
+          <t>Centro Multidisciplinar de Angicos</t>
+        </is>
       </c>
       <c r="G27" s="9" t="s">
         <v>174</v>
@@ -3451,8 +3461,10 @@
       <c r="E37" t="s">
         <v>332</v>
       </c>
-      <c r="F37" s="1" t="s">
-        <v>153</v>
+      <c r="F37" s="1" t="inlineStr">
+        <is>
+          <t>Centro Multidisciplinar de Angicos</t>
+        </is>
       </c>
       <c r="G37" s="1" t="s">
         <v>154</v>
@@ -33610,8 +33622,10 @@
       </c>
     </row>
     <row r="6" spans="1:6" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="18" t="s">
-        <v>341</v>
+      <c r="A6" s="18" t="inlineStr">
+        <is>
+          <t>centro-multidisciplinar-de-angicos</t>
+        </is>
       </c>
       <c r="B6" s="18" t="s">
         <v>341</v>

</xml_diff>

<commit_message>
Patch: substituição da foto de Leandro e mudança de v para V em Visualização em tela cheia.
</commit_message>
<xml_diff>
--- a/Corpo Administrativo.xlsx
+++ b/Corpo Administrativo.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\leanm\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\leanm\OneDrive\Documentos\Dev\Studies\corpo_administrativo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E277FACD-87C7-4A88-9BF6-3B2D39A977D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84C767FF-1684-4CC2-BB96-2F10342CCB88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -487,9 +487,6 @@
     <t>Alexzuza@ufersa.edu.br</t>
   </si>
   <si>
-    <t>Direção</t>
-  </si>
-  <si>
     <t>Secretaria Administrativa</t>
   </si>
   <si>
@@ -754,9 +751,6 @@
     <t>2d2c7bbc-3d80-50d5-b30a-045c72a563fc</t>
   </si>
   <si>
-    <t>Leandro.jpg</t>
-  </si>
-  <si>
     <t>c6253b3f-d948-58e9-8cc2-e9f42125116f</t>
   </si>
   <si>
@@ -1172,6 +1166,12 @@
   </si>
   <si>
     <t>21/09</t>
+  </si>
+  <si>
+    <t>centro-multidisciplinar-de-angicos</t>
+  </si>
+  <si>
+    <t>Leandro.png</t>
   </si>
 </sst>
 </file>
@@ -1299,7 +1299,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -1325,8 +1325,6 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hiperlink" xfId="1" builtinId="8"/>
@@ -1571,7 +1569,7 @@
         <v>3</v>
       </c>
       <c r="E1" s="12" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="F1" s="6" t="s">
         <v>4</v>
@@ -1589,10 +1587,10 @@
         <v>8</v>
       </c>
       <c r="K1" s="7" t="s">
+        <v>174</v>
+      </c>
+      <c r="L1" s="7" t="s">
         <v>175</v>
-      </c>
-      <c r="L1" s="7" t="s">
-        <v>176</v>
       </c>
       <c r="M1" s="1"/>
       <c r="N1" s="1"/>
@@ -1626,7 +1624,7 @@
         <v>46</v>
       </c>
       <c r="E2" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="F2" t="s">
         <v>47</v>
@@ -1635,7 +1633,7 @@
         <v>48</v>
       </c>
       <c r="H2" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="I2" t="s">
         <v>15</v>
@@ -1644,10 +1642,10 @@
         <v>15</v>
       </c>
       <c r="K2" t="s">
+        <v>192</v>
+      </c>
+      <c r="L2" t="s">
         <v>193</v>
-      </c>
-      <c r="L2" t="s">
-        <v>194</v>
       </c>
     </row>
     <row r="3" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1664,7 +1662,7 @@
         <v>12</v>
       </c>
       <c r="E3" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="F3" t="s">
         <v>13</v>
@@ -1673,7 +1671,7 @@
         <v>14</v>
       </c>
       <c r="H3" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="I3" t="s">
         <v>15</v>
@@ -1682,10 +1680,10 @@
         <v>15</v>
       </c>
       <c r="K3" t="s">
+        <v>176</v>
+      </c>
+      <c r="L3" t="s">
         <v>177</v>
-      </c>
-      <c r="L3" t="s">
-        <v>178</v>
       </c>
     </row>
     <row r="4" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1702,7 +1700,7 @@
         <v>52</v>
       </c>
       <c r="E4" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="F4" t="s">
         <v>47</v>
@@ -1711,7 +1709,7 @@
         <v>48</v>
       </c>
       <c r="H4" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="I4" t="s">
         <v>15</v>
@@ -1720,10 +1718,10 @@
         <v>15</v>
       </c>
       <c r="K4" t="s">
+        <v>194</v>
+      </c>
+      <c r="L4" t="s">
         <v>195</v>
-      </c>
-      <c r="L4" t="s">
-        <v>196</v>
       </c>
     </row>
     <row r="5" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1740,7 +1738,7 @@
         <v>89</v>
       </c>
       <c r="E5" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="F5" t="s">
         <v>90</v>
@@ -1749,7 +1747,7 @@
         <v>14</v>
       </c>
       <c r="H5" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="I5" t="s">
         <v>15</v>
@@ -1758,10 +1756,10 @@
         <v>15</v>
       </c>
       <c r="K5" t="s">
+        <v>214</v>
+      </c>
+      <c r="L5" t="s">
         <v>215</v>
-      </c>
-      <c r="L5" t="s">
-        <v>216</v>
       </c>
     </row>
     <row r="6" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1778,7 +1776,7 @@
         <v>93</v>
       </c>
       <c r="E6" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="F6" t="s">
         <v>90</v>
@@ -1787,7 +1785,7 @@
         <v>14</v>
       </c>
       <c r="H6" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="I6" t="s">
         <v>15</v>
@@ -1796,10 +1794,10 @@
         <v>15</v>
       </c>
       <c r="K6" t="s">
+        <v>216</v>
+      </c>
+      <c r="L6" t="s">
         <v>217</v>
-      </c>
-      <c r="L6" t="s">
-        <v>218</v>
       </c>
     </row>
     <row r="7" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1816,7 +1814,7 @@
         <v>106</v>
       </c>
       <c r="E7" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="F7" t="s">
         <v>107</v>
@@ -1825,7 +1823,7 @@
         <v>108</v>
       </c>
       <c r="H7" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
       <c r="I7" t="s">
         <v>15</v>
@@ -1834,10 +1832,10 @@
         <v>15</v>
       </c>
       <c r="K7" t="s">
+        <v>224</v>
+      </c>
+      <c r="L7" t="s">
         <v>225</v>
-      </c>
-      <c r="L7" t="s">
-        <v>226</v>
       </c>
     </row>
     <row r="8" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1854,7 +1852,7 @@
         <v>19</v>
       </c>
       <c r="E8" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="F8" t="s">
         <v>13</v>
@@ -1863,7 +1861,7 @@
         <v>14</v>
       </c>
       <c r="H8" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="I8" t="s">
         <v>15</v>
@@ -1872,10 +1870,10 @@
         <v>15</v>
       </c>
       <c r="K8" t="s">
+        <v>178</v>
+      </c>
+      <c r="L8" t="s">
         <v>179</v>
-      </c>
-      <c r="L8" t="s">
-        <v>180</v>
       </c>
     </row>
     <row r="9" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1892,7 +1890,7 @@
         <v>111</v>
       </c>
       <c r="E9" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="F9" t="s">
         <v>107</v>
@@ -1901,7 +1899,7 @@
         <v>112</v>
       </c>
       <c r="H9" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
       <c r="I9" t="s">
         <v>15</v>
@@ -1910,7 +1908,7 @@
         <v>15</v>
       </c>
       <c r="L9" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
     </row>
     <row r="10" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1927,7 +1925,7 @@
         <v>115</v>
       </c>
       <c r="E10" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="F10" t="s">
         <v>107</v>
@@ -1936,7 +1934,7 @@
         <v>116</v>
       </c>
       <c r="H10" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="I10" t="s">
         <v>15</v>
@@ -1945,10 +1943,10 @@
         <v>15</v>
       </c>
       <c r="K10" t="s">
+        <v>227</v>
+      </c>
+      <c r="L10" t="s">
         <v>228</v>
-      </c>
-      <c r="L10" t="s">
-        <v>229</v>
       </c>
     </row>
     <row r="11" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1965,7 +1963,7 @@
         <v>119</v>
       </c>
       <c r="E11" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="F11" t="s">
         <v>107</v>
@@ -1974,7 +1972,7 @@
         <v>108</v>
       </c>
       <c r="H11" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="I11" t="s">
         <v>15</v>
@@ -1983,10 +1981,10 @@
         <v>15</v>
       </c>
       <c r="K11" t="s">
+        <v>229</v>
+      </c>
+      <c r="L11" t="s">
         <v>230</v>
-      </c>
-      <c r="L11" t="s">
-        <v>231</v>
       </c>
     </row>
     <row r="12" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -2003,7 +2001,7 @@
         <v>96</v>
       </c>
       <c r="E12" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="F12" t="s">
         <v>90</v>
@@ -2012,7 +2010,7 @@
         <v>97</v>
       </c>
       <c r="H12" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="I12" t="s">
         <v>15</v>
@@ -2021,10 +2019,10 @@
         <v>15</v>
       </c>
       <c r="K12" t="s">
+        <v>218</v>
+      </c>
+      <c r="L12" t="s">
         <v>219</v>
-      </c>
-      <c r="L12" t="s">
-        <v>220</v>
       </c>
     </row>
     <row r="13" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -2041,7 +2039,7 @@
         <v>56</v>
       </c>
       <c r="E13" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="F13" t="s">
         <v>47</v>
@@ -2050,7 +2048,7 @@
         <v>48</v>
       </c>
       <c r="H13" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="I13" t="s">
         <v>15</v>
@@ -2059,10 +2057,10 @@
         <v>15</v>
       </c>
       <c r="K13" t="s">
+        <v>196</v>
+      </c>
+      <c r="L13" t="s">
         <v>197</v>
-      </c>
-      <c r="L13" t="s">
-        <v>198</v>
       </c>
     </row>
     <row r="14" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -2079,7 +2077,7 @@
         <v>59</v>
       </c>
       <c r="E14" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="F14" t="s">
         <v>47</v>
@@ -2088,7 +2086,7 @@
         <v>60</v>
       </c>
       <c r="H14" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="I14" t="s">
         <v>15</v>
@@ -2097,10 +2095,10 @@
         <v>15</v>
       </c>
       <c r="K14" t="s">
+        <v>198</v>
+      </c>
+      <c r="L14" t="s">
         <v>199</v>
-      </c>
-      <c r="L14" t="s">
-        <v>200</v>
       </c>
     </row>
     <row r="15" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -2117,18 +2115,16 @@
         <v>152</v>
       </c>
       <c r="E15" t="s">
-        <v>332</v>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>Centro Multidisciplinar de Angicos</t>
-        </is>
+        <v>330</v>
+      </c>
+      <c r="F15" t="s">
+        <v>339</v>
       </c>
       <c r="G15" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="H15" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="I15" t="s">
         <v>15</v>
@@ -2137,38 +2133,36 @@
         <v>15</v>
       </c>
       <c r="K15" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="L15" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
     </row>
     <row r="16" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
+        <v>161</v>
+      </c>
+      <c r="B16" t="s">
         <v>162</v>
-      </c>
-      <c r="B16" t="s">
-        <v>163</v>
       </c>
       <c r="C16" t="s">
         <v>70</v>
       </c>
       <c r="D16" t="s">
+        <v>164</v>
+      </c>
+      <c r="E16" t="s">
+        <v>328</v>
+      </c>
+      <c r="F16" t="s">
+        <v>339</v>
+      </c>
+      <c r="G16" t="s">
         <v>165</v>
       </c>
-      <c r="E16" t="s">
-        <v>330</v>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>Centro Multidisciplinar de Angicos</t>
-        </is>
-      </c>
-      <c r="G16" t="s">
-        <v>166</v>
-      </c>
       <c r="H16" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="I16" t="s">
         <v>15</v>
@@ -2177,38 +2171,36 @@
         <v>15</v>
       </c>
       <c r="K16" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="L16" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
     </row>
     <row r="17" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
+        <v>166</v>
+      </c>
+      <c r="B17" t="s">
         <v>167</v>
-      </c>
-      <c r="B17" t="s">
-        <v>168</v>
       </c>
       <c r="C17" t="s">
         <v>70</v>
       </c>
       <c r="D17" t="s">
+        <v>168</v>
+      </c>
+      <c r="E17" t="s">
+        <v>328</v>
+      </c>
+      <c r="F17" t="s">
+        <v>339</v>
+      </c>
+      <c r="G17" t="s">
         <v>169</v>
       </c>
-      <c r="E17" t="s">
-        <v>330</v>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>Centro Multidisciplinar de Angicos</t>
-        </is>
-      </c>
-      <c r="G17" t="s">
-        <v>170</v>
-      </c>
       <c r="H17" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
       <c r="I17" t="s">
         <v>15</v>
@@ -2217,10 +2209,10 @@
         <v>15</v>
       </c>
       <c r="K17" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="L17" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
     </row>
     <row r="18" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -2237,7 +2229,7 @@
         <v>22</v>
       </c>
       <c r="E18" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="F18" t="s">
         <v>13</v>
@@ -2246,7 +2238,7 @@
         <v>14</v>
       </c>
       <c r="H18" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="I18" t="s">
         <v>15</v>
@@ -2255,10 +2247,10 @@
         <v>15</v>
       </c>
       <c r="K18" t="s">
+        <v>180</v>
+      </c>
+      <c r="L18" t="s">
         <v>181</v>
-      </c>
-      <c r="L18" t="s">
-        <v>182</v>
       </c>
     </row>
     <row r="19" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -2275,7 +2267,7 @@
         <v>122</v>
       </c>
       <c r="E19" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="F19" t="s">
         <v>107</v>
@@ -2284,7 +2276,7 @@
         <v>116</v>
       </c>
       <c r="H19" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="I19" t="s">
         <v>15</v>
@@ -2293,10 +2285,10 @@
         <v>15</v>
       </c>
       <c r="K19" t="s">
+        <v>231</v>
+      </c>
+      <c r="L19" t="s">
         <v>232</v>
-      </c>
-      <c r="L19" t="s">
-        <v>233</v>
       </c>
     </row>
     <row r="20" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -2313,7 +2305,7 @@
         <v>26</v>
       </c>
       <c r="E20" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="F20" t="s">
         <v>13</v>
@@ -2322,7 +2314,7 @@
         <v>27</v>
       </c>
       <c r="H20" t="s">
-        <v>381</v>
+        <v>379</v>
       </c>
       <c r="I20" t="s">
         <v>15</v>
@@ -2331,10 +2323,10 @@
         <v>15</v>
       </c>
       <c r="K20" t="s">
+        <v>182</v>
+      </c>
+      <c r="L20" t="s">
         <v>183</v>
-      </c>
-      <c r="L20" t="s">
-        <v>184</v>
       </c>
     </row>
     <row r="21" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -2351,7 +2343,7 @@
         <v>126</v>
       </c>
       <c r="E21" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="F21" t="s">
         <v>107</v>
@@ -2360,7 +2352,7 @@
         <v>127</v>
       </c>
       <c r="H21" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="I21" t="s">
         <v>15</v>
@@ -2369,10 +2361,10 @@
         <v>15</v>
       </c>
       <c r="K21" t="s">
+        <v>233</v>
+      </c>
+      <c r="L21" t="s">
         <v>234</v>
-      </c>
-      <c r="L21" t="s">
-        <v>235</v>
       </c>
     </row>
     <row r="22" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -2389,7 +2381,7 @@
         <v>64</v>
       </c>
       <c r="E22" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="F22" t="s">
         <v>47</v>
@@ -2398,7 +2390,7 @@
         <v>48</v>
       </c>
       <c r="H22" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="I22" t="s">
         <v>15</v>
@@ -2407,10 +2399,10 @@
         <v>15</v>
       </c>
       <c r="K22" t="s">
+        <v>200</v>
+      </c>
+      <c r="L22" t="s">
         <v>201</v>
-      </c>
-      <c r="L22" t="s">
-        <v>202</v>
       </c>
     </row>
     <row r="23" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -2427,7 +2419,7 @@
         <v>31</v>
       </c>
       <c r="E23" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="F23" t="s">
         <v>13</v>
@@ -2436,7 +2428,7 @@
         <v>14</v>
       </c>
       <c r="H23" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="I23" t="s">
         <v>15</v>
@@ -2445,10 +2437,10 @@
         <v>15</v>
       </c>
       <c r="K23" t="s">
+        <v>184</v>
+      </c>
+      <c r="L23" t="s">
         <v>185</v>
-      </c>
-      <c r="L23" t="s">
-        <v>186</v>
       </c>
     </row>
     <row r="24" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -2465,7 +2457,7 @@
         <v>130</v>
       </c>
       <c r="E24" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="F24" t="s">
         <v>107</v>
@@ -2474,7 +2466,7 @@
         <v>108</v>
       </c>
       <c r="H24" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="I24" t="s">
         <v>15</v>
@@ -2483,10 +2475,10 @@
         <v>15</v>
       </c>
       <c r="K24" t="s">
+        <v>235</v>
+      </c>
+      <c r="L24" t="s">
         <v>236</v>
-      </c>
-      <c r="L24" t="s">
-        <v>237</v>
       </c>
     </row>
     <row r="25" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -2503,7 +2495,7 @@
         <v>67</v>
       </c>
       <c r="E25" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="F25" t="s">
         <v>47</v>
@@ -2512,7 +2504,7 @@
         <v>48</v>
       </c>
       <c r="H25" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
       <c r="I25" t="s">
         <v>15</v>
@@ -2521,38 +2513,36 @@
         <v>15</v>
       </c>
       <c r="K25" t="s">
+        <v>202</v>
+      </c>
+      <c r="L25" t="s">
         <v>203</v>
-      </c>
-      <c r="L25" t="s">
-        <v>204</v>
       </c>
     </row>
     <row r="26" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
+        <v>154</v>
+      </c>
+      <c r="B26" t="s">
         <v>155</v>
-      </c>
-      <c r="B26" t="s">
-        <v>156</v>
       </c>
       <c r="C26" t="s">
         <v>25</v>
       </c>
       <c r="D26" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="E26" t="s">
-        <v>332</v>
-      </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>Centro Multidisciplinar de Angicos</t>
-        </is>
+        <v>330</v>
+      </c>
+      <c r="F26" t="s">
+        <v>339</v>
       </c>
       <c r="G26" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="H26" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="I26" t="s">
         <v>15</v>
@@ -2561,38 +2551,36 @@
         <v>15</v>
       </c>
       <c r="K26" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="L26" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
     </row>
     <row r="27" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
+        <v>170</v>
+      </c>
+      <c r="B27" t="s">
         <v>171</v>
-      </c>
-      <c r="B27" t="s">
-        <v>172</v>
       </c>
       <c r="C27" t="s">
         <v>25</v>
       </c>
       <c r="D27" t="s">
+        <v>172</v>
+      </c>
+      <c r="E27" t="s">
+        <v>330</v>
+      </c>
+      <c r="F27" t="s">
+        <v>339</v>
+      </c>
+      <c r="G27" t="s">
         <v>173</v>
       </c>
-      <c r="E27" t="s">
-        <v>332</v>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>Centro Multidisciplinar de Angicos</t>
-        </is>
-      </c>
-      <c r="G27" t="s">
-        <v>174</v>
-      </c>
       <c r="H27" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="I27" t="s">
         <v>15</v>
@@ -2601,10 +2589,10 @@
         <v>15</v>
       </c>
       <c r="K27" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="L27" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
     </row>
     <row r="28" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -2621,7 +2609,7 @@
         <v>35</v>
       </c>
       <c r="E28" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="F28" t="s">
         <v>13</v>
@@ -2630,7 +2618,7 @@
         <v>14</v>
       </c>
       <c r="H28" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="I28" t="s">
         <v>15</v>
@@ -2639,10 +2627,10 @@
         <v>15</v>
       </c>
       <c r="K28" t="s">
+        <v>186</v>
+      </c>
+      <c r="L28" t="s">
         <v>187</v>
-      </c>
-      <c r="L28" t="s">
-        <v>188</v>
       </c>
     </row>
     <row r="29" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -2659,7 +2647,7 @@
         <v>71</v>
       </c>
       <c r="E29" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="F29" t="s">
         <v>47</v>
@@ -2668,7 +2656,7 @@
         <v>72</v>
       </c>
       <c r="H29" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="I29" t="s">
         <v>15</v>
@@ -2677,10 +2665,10 @@
         <v>15</v>
       </c>
       <c r="K29" t="s">
+        <v>204</v>
+      </c>
+      <c r="L29" t="s">
         <v>205</v>
-      </c>
-      <c r="L29" t="s">
-        <v>206</v>
       </c>
     </row>
     <row r="30" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -2697,7 +2685,7 @@
         <v>134</v>
       </c>
       <c r="E30" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="F30" t="s">
         <v>107</v>
@@ -2706,7 +2694,7 @@
         <v>97</v>
       </c>
       <c r="H30" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="I30" t="s">
         <v>15</v>
@@ -2715,10 +2703,10 @@
         <v>15</v>
       </c>
       <c r="K30" t="s">
+        <v>237</v>
+      </c>
+      <c r="L30" t="s">
         <v>238</v>
-      </c>
-      <c r="L30" t="s">
-        <v>239</v>
       </c>
     </row>
     <row r="31" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -2735,7 +2723,7 @@
         <v>100</v>
       </c>
       <c r="E31" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="F31" t="s">
         <v>90</v>
@@ -2744,7 +2732,7 @@
         <v>14</v>
       </c>
       <c r="H31" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="I31" t="s">
         <v>15</v>
@@ -2753,10 +2741,10 @@
         <v>15</v>
       </c>
       <c r="K31" t="s">
+        <v>220</v>
+      </c>
+      <c r="L31" t="s">
         <v>221</v>
-      </c>
-      <c r="L31" t="s">
-        <v>222</v>
       </c>
     </row>
     <row r="32" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -2773,7 +2761,7 @@
         <v>75</v>
       </c>
       <c r="E32" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="F32" t="s">
         <v>47</v>
@@ -2782,7 +2770,7 @@
         <v>72</v>
       </c>
       <c r="H32" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="I32" t="s">
         <v>15</v>
@@ -2791,10 +2779,10 @@
         <v>15</v>
       </c>
       <c r="K32" t="s">
+        <v>206</v>
+      </c>
+      <c r="L32" t="s">
         <v>207</v>
-      </c>
-      <c r="L32" t="s">
-        <v>208</v>
       </c>
     </row>
     <row r="33" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -2811,7 +2799,7 @@
         <v>78</v>
       </c>
       <c r="E33" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="F33" t="s">
         <v>47</v>
@@ -2820,7 +2808,7 @@
         <v>48</v>
       </c>
       <c r="H33" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="I33" t="s">
         <v>15</v>
@@ -2829,10 +2817,10 @@
         <v>15</v>
       </c>
       <c r="K33" t="s">
+        <v>208</v>
+      </c>
+      <c r="L33" t="s">
         <v>209</v>
-      </c>
-      <c r="L33" t="s">
-        <v>210</v>
       </c>
     </row>
     <row r="34" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -2849,7 +2837,7 @@
         <v>38</v>
       </c>
       <c r="E34" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="F34" t="s">
         <v>13</v>
@@ -2858,7 +2846,7 @@
         <v>14</v>
       </c>
       <c r="H34" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="I34" t="s">
         <v>15</v>
@@ -2867,10 +2855,10 @@
         <v>15</v>
       </c>
       <c r="K34" t="s">
+        <v>188</v>
+      </c>
+      <c r="L34" t="s">
         <v>189</v>
-      </c>
-      <c r="L34" t="s">
-        <v>190</v>
       </c>
     </row>
     <row r="35" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -2887,7 +2875,7 @@
         <v>137</v>
       </c>
       <c r="E35" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="F35" t="s">
         <v>107</v>
@@ -2896,7 +2884,7 @@
         <v>138</v>
       </c>
       <c r="H35" t="s">
-        <v>377</v>
+        <v>375</v>
       </c>
       <c r="I35" t="s">
         <v>15</v>
@@ -2905,10 +2893,10 @@
         <v>15</v>
       </c>
       <c r="K35" t="s">
+        <v>239</v>
+      </c>
+      <c r="L35" t="s">
         <v>240</v>
-      </c>
-      <c r="L35" t="s">
-        <v>241</v>
       </c>
     </row>
     <row r="36" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -2925,7 +2913,7 @@
         <v>42</v>
       </c>
       <c r="E36" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="F36" t="s">
         <v>13</v>
@@ -2934,7 +2922,7 @@
         <v>14</v>
       </c>
       <c r="H36" t="s">
-        <v>378</v>
+        <v>376</v>
       </c>
       <c r="I36" t="s">
         <v>15</v>
@@ -2943,38 +2931,36 @@
         <v>15</v>
       </c>
       <c r="K36" t="s">
+        <v>190</v>
+      </c>
+      <c r="L36" t="s">
         <v>191</v>
-      </c>
-      <c r="L36" t="s">
-        <v>192</v>
       </c>
     </row>
     <row r="37" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
+        <v>157</v>
+      </c>
+      <c r="B37" t="s">
         <v>158</v>
-      </c>
-      <c r="B37" t="s">
-        <v>159</v>
       </c>
       <c r="C37" t="s">
         <v>25</v>
       </c>
       <c r="D37" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="E37" t="s">
-        <v>332</v>
-      </c>
-      <c r="F37" t="inlineStr">
-        <is>
-          <t>Centro Multidisciplinar de Angicos</t>
-        </is>
+        <v>330</v>
+      </c>
+      <c r="F37" t="s">
+        <v>339</v>
       </c>
       <c r="G37" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="H37" t="s">
-        <v>379</v>
+        <v>377</v>
       </c>
       <c r="I37" t="s">
         <v>15</v>
@@ -2983,10 +2969,10 @@
         <v>15</v>
       </c>
       <c r="K37" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="L37" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
     </row>
     <row r="38" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3003,7 +2989,7 @@
         <v>81</v>
       </c>
       <c r="E38" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="F38" t="s">
         <v>47</v>
@@ -3012,7 +2998,7 @@
         <v>60</v>
       </c>
       <c r="H38" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="I38" t="s">
         <v>15</v>
@@ -3021,10 +3007,10 @@
         <v>15</v>
       </c>
       <c r="K38" t="s">
+        <v>210</v>
+      </c>
+      <c r="L38" t="s">
         <v>211</v>
-      </c>
-      <c r="L38" t="s">
-        <v>212</v>
       </c>
     </row>
     <row r="39" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3041,7 +3027,7 @@
         <v>141</v>
       </c>
       <c r="E39" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="F39" t="s">
         <v>107</v>
@@ -3050,7 +3036,7 @@
         <v>138</v>
       </c>
       <c r="H39" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="I39" t="s">
         <v>15</v>
@@ -3059,10 +3045,10 @@
         <v>15</v>
       </c>
       <c r="K39" t="s">
-        <v>242</v>
+        <v>381</v>
       </c>
       <c r="L39" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
     </row>
     <row r="40" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3073,13 +3059,13 @@
         <v>143</v>
       </c>
       <c r="C40" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D40" t="s">
         <v>144</v>
       </c>
       <c r="E40" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="F40" t="s">
         <v>107</v>
@@ -3088,7 +3074,7 @@
         <v>145</v>
       </c>
       <c r="H40" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="I40" t="s">
         <v>15</v>
@@ -3097,10 +3083,10 @@
         <v>15</v>
       </c>
       <c r="K40" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="L40" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
     </row>
     <row r="41" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3111,13 +3097,13 @@
         <v>147</v>
       </c>
       <c r="C41" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="D41" t="s">
         <v>148</v>
       </c>
       <c r="E41" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="F41" t="s">
         <v>107</v>
@@ -3126,7 +3112,7 @@
         <v>127</v>
       </c>
       <c r="H41" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="I41" t="s">
         <v>15</v>
@@ -3135,10 +3121,10 @@
         <v>15</v>
       </c>
       <c r="K41" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="L41" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
     </row>
     <row r="42" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3155,7 +3141,7 @@
         <v>103</v>
       </c>
       <c r="E42" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="F42" t="s">
         <v>90</v>
@@ -3164,7 +3150,7 @@
         <v>14</v>
       </c>
       <c r="H42" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
       <c r="I42" t="s">
         <v>15</v>
@@ -3173,10 +3159,10 @@
         <v>15</v>
       </c>
       <c r="K42" t="s">
+        <v>222</v>
+      </c>
+      <c r="L42" t="s">
         <v>223</v>
-      </c>
-      <c r="L42" t="s">
-        <v>224</v>
       </c>
     </row>
     <row r="43" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3193,7 +3179,7 @@
         <v>85</v>
       </c>
       <c r="E43" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="F43" t="s">
         <v>47</v>
@@ -3202,7 +3188,7 @@
         <v>72</v>
       </c>
       <c r="H43" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="I43" t="s">
         <v>15</v>
@@ -3211,10 +3197,10 @@
         <v>15</v>
       </c>
       <c r="K43" t="s">
+        <v>212</v>
+      </c>
+      <c r="L43" t="s">
         <v>213</v>
-      </c>
-      <c r="L43" t="s">
-        <v>214</v>
       </c>
     </row>
     <row r="44" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -3227,7 +3213,7 @@
       <c r="E46" s="2"/>
       <c r="F46" s="2"/>
       <c r="G46" s="2"/>
-      <c r="H46" s="15"/>
+      <c r="H46" s="2"/>
       <c r="I46" s="2"/>
       <c r="J46" s="2"/>
       <c r="K46" s="2"/>
@@ -3258,7 +3244,7 @@
       <c r="E47" s="3"/>
       <c r="F47" s="3"/>
       <c r="G47" s="3"/>
-      <c r="H47" s="16"/>
+      <c r="H47" s="3"/>
       <c r="I47" s="3"/>
       <c r="J47" s="3"/>
       <c r="K47" s="3"/>
@@ -3289,7 +3275,7 @@
       <c r="E48" s="2"/>
       <c r="F48" s="2"/>
       <c r="G48" s="2"/>
-      <c r="H48" s="15"/>
+      <c r="H48" s="2"/>
       <c r="I48" s="2"/>
       <c r="J48" s="2"/>
       <c r="K48" s="2"/>
@@ -3320,7 +3306,7 @@
       <c r="E49" s="3"/>
       <c r="F49" s="3"/>
       <c r="G49" s="3"/>
-      <c r="H49" s="16"/>
+      <c r="H49" s="3"/>
       <c r="I49" s="3"/>
       <c r="J49" s="3"/>
       <c r="K49" s="3"/>
@@ -3351,7 +3337,7 @@
       <c r="E50" s="2"/>
       <c r="F50" s="2"/>
       <c r="G50" s="2"/>
-      <c r="H50" s="15"/>
+      <c r="H50" s="2"/>
       <c r="I50" s="2"/>
       <c r="J50" s="2"/>
       <c r="K50" s="2"/>
@@ -3382,7 +3368,7 @@
       <c r="E51" s="3"/>
       <c r="F51" s="3"/>
       <c r="G51" s="3"/>
-      <c r="H51" s="16"/>
+      <c r="H51" s="3"/>
       <c r="I51" s="3"/>
       <c r="J51" s="3"/>
       <c r="K51" s="3"/>
@@ -3413,7 +3399,7 @@
       <c r="E52" s="2"/>
       <c r="F52" s="2"/>
       <c r="G52" s="2"/>
-      <c r="H52" s="15"/>
+      <c r="H52" s="2"/>
       <c r="I52" s="2"/>
       <c r="J52" s="2"/>
       <c r="K52" s="2"/>
@@ -3444,7 +3430,7 @@
       <c r="E53" s="3"/>
       <c r="F53" s="3"/>
       <c r="G53" s="3"/>
-      <c r="H53" s="16"/>
+      <c r="H53" s="3"/>
       <c r="I53" s="3"/>
       <c r="J53" s="3"/>
       <c r="K53" s="3"/>
@@ -3475,7 +3461,7 @@
       <c r="E54" s="2"/>
       <c r="F54" s="2"/>
       <c r="G54" s="2"/>
-      <c r="H54" s="15"/>
+      <c r="H54" s="2"/>
       <c r="I54" s="2"/>
       <c r="J54" s="2"/>
       <c r="K54" s="2"/>
@@ -3506,7 +3492,7 @@
       <c r="E55" s="3"/>
       <c r="F55" s="3"/>
       <c r="G55" s="3"/>
-      <c r="H55" s="16"/>
+      <c r="H55" s="3"/>
       <c r="I55" s="3"/>
       <c r="J55" s="3"/>
       <c r="K55" s="3"/>
@@ -3537,7 +3523,7 @@
       <c r="E56" s="2"/>
       <c r="F56" s="2"/>
       <c r="G56" s="2"/>
-      <c r="H56" s="15"/>
+      <c r="H56" s="2"/>
       <c r="I56" s="2"/>
       <c r="J56" s="2"/>
       <c r="K56" s="2"/>
@@ -3568,7 +3554,7 @@
       <c r="E57" s="3"/>
       <c r="F57" s="3"/>
       <c r="G57" s="3"/>
-      <c r="H57" s="16"/>
+      <c r="H57" s="3"/>
       <c r="I57" s="3"/>
       <c r="J57" s="3"/>
       <c r="K57" s="3"/>
@@ -3599,7 +3585,7 @@
       <c r="E58" s="2"/>
       <c r="F58" s="2"/>
       <c r="G58" s="2"/>
-      <c r="H58" s="15"/>
+      <c r="H58" s="2"/>
       <c r="I58" s="2"/>
       <c r="J58" s="2"/>
       <c r="K58" s="2"/>
@@ -3630,7 +3616,7 @@
       <c r="E59" s="3"/>
       <c r="F59" s="3"/>
       <c r="G59" s="3"/>
-      <c r="H59" s="16"/>
+      <c r="H59" s="3"/>
       <c r="I59" s="3"/>
       <c r="J59" s="3"/>
       <c r="K59" s="3"/>
@@ -3661,7 +3647,7 @@
       <c r="E60" s="2"/>
       <c r="F60" s="2"/>
       <c r="G60" s="2"/>
-      <c r="H60" s="15"/>
+      <c r="H60" s="2"/>
       <c r="I60" s="2"/>
       <c r="J60" s="2"/>
       <c r="K60" s="2"/>
@@ -3692,7 +3678,7 @@
       <c r="E61" s="3"/>
       <c r="F61" s="3"/>
       <c r="G61" s="3"/>
-      <c r="H61" s="16"/>
+      <c r="H61" s="3"/>
       <c r="I61" s="3"/>
       <c r="J61" s="3"/>
       <c r="K61" s="3"/>
@@ -3723,7 +3709,7 @@
       <c r="E62" s="2"/>
       <c r="F62" s="2"/>
       <c r="G62" s="2"/>
-      <c r="H62" s="15"/>
+      <c r="H62" s="2"/>
       <c r="I62" s="2"/>
       <c r="J62" s="2"/>
       <c r="K62" s="2"/>
@@ -3754,7 +3740,7 @@
       <c r="E63" s="3"/>
       <c r="F63" s="3"/>
       <c r="G63" s="3"/>
-      <c r="H63" s="16"/>
+      <c r="H63" s="3"/>
       <c r="I63" s="3"/>
       <c r="J63" s="3"/>
       <c r="K63" s="3"/>
@@ -3785,7 +3771,7 @@
       <c r="E64" s="2"/>
       <c r="F64" s="2"/>
       <c r="G64" s="2"/>
-      <c r="H64" s="15"/>
+      <c r="H64" s="2"/>
       <c r="I64" s="2"/>
       <c r="J64" s="2"/>
       <c r="K64" s="2"/>
@@ -3816,7 +3802,7 @@
       <c r="E65" s="3"/>
       <c r="F65" s="3"/>
       <c r="G65" s="3"/>
-      <c r="H65" s="16"/>
+      <c r="H65" s="3"/>
       <c r="I65" s="3"/>
       <c r="J65" s="3"/>
       <c r="K65" s="3"/>
@@ -3847,7 +3833,7 @@
       <c r="E66" s="2"/>
       <c r="F66" s="2"/>
       <c r="G66" s="2"/>
-      <c r="H66" s="15"/>
+      <c r="H66" s="2"/>
       <c r="I66" s="2"/>
       <c r="J66" s="2"/>
       <c r="K66" s="2"/>
@@ -3878,7 +3864,7 @@
       <c r="E67" s="3"/>
       <c r="F67" s="3"/>
       <c r="G67" s="3"/>
-      <c r="H67" s="16"/>
+      <c r="H67" s="3"/>
       <c r="I67" s="3"/>
       <c r="J67" s="3"/>
       <c r="K67" s="3"/>
@@ -3909,7 +3895,7 @@
       <c r="E68" s="2"/>
       <c r="F68" s="2"/>
       <c r="G68" s="2"/>
-      <c r="H68" s="15"/>
+      <c r="H68" s="2"/>
       <c r="I68" s="2"/>
       <c r="J68" s="2"/>
       <c r="K68" s="2"/>
@@ -3940,7 +3926,7 @@
       <c r="E69" s="3"/>
       <c r="F69" s="3"/>
       <c r="G69" s="3"/>
-      <c r="H69" s="16"/>
+      <c r="H69" s="3"/>
       <c r="I69" s="3"/>
       <c r="J69" s="3"/>
       <c r="K69" s="3"/>
@@ -3971,7 +3957,7 @@
       <c r="E70" s="2"/>
       <c r="F70" s="2"/>
       <c r="G70" s="2"/>
-      <c r="H70" s="15"/>
+      <c r="H70" s="2"/>
       <c r="I70" s="2"/>
       <c r="J70" s="2"/>
       <c r="K70" s="2"/>
@@ -4002,7 +3988,7 @@
       <c r="E71" s="3"/>
       <c r="F71" s="3"/>
       <c r="G71" s="3"/>
-      <c r="H71" s="16"/>
+      <c r="H71" s="3"/>
       <c r="I71" s="3"/>
       <c r="J71" s="3"/>
       <c r="K71" s="3"/>
@@ -4033,7 +4019,7 @@
       <c r="E72" s="2"/>
       <c r="F72" s="2"/>
       <c r="G72" s="2"/>
-      <c r="H72" s="15"/>
+      <c r="H72" s="2"/>
       <c r="I72" s="2"/>
       <c r="J72" s="2"/>
       <c r="K72" s="2"/>
@@ -4064,7 +4050,7 @@
       <c r="E73" s="3"/>
       <c r="F73" s="3"/>
       <c r="G73" s="3"/>
-      <c r="H73" s="16"/>
+      <c r="H73" s="3"/>
       <c r="I73" s="3"/>
       <c r="J73" s="3"/>
       <c r="K73" s="3"/>
@@ -4095,7 +4081,7 @@
       <c r="E74" s="2"/>
       <c r="F74" s="2"/>
       <c r="G74" s="2"/>
-      <c r="H74" s="15"/>
+      <c r="H74" s="2"/>
       <c r="I74" s="2"/>
       <c r="J74" s="2"/>
       <c r="K74" s="2"/>
@@ -4126,7 +4112,7 @@
       <c r="E75" s="3"/>
       <c r="F75" s="3"/>
       <c r="G75" s="3"/>
-      <c r="H75" s="16"/>
+      <c r="H75" s="3"/>
       <c r="I75" s="3"/>
       <c r="J75" s="3"/>
       <c r="K75" s="3"/>
@@ -4157,7 +4143,7 @@
       <c r="E76" s="2"/>
       <c r="F76" s="2"/>
       <c r="G76" s="2"/>
-      <c r="H76" s="15"/>
+      <c r="H76" s="2"/>
       <c r="I76" s="2"/>
       <c r="J76" s="2"/>
       <c r="K76" s="2"/>
@@ -4188,7 +4174,7 @@
       <c r="E77" s="3"/>
       <c r="F77" s="3"/>
       <c r="G77" s="3"/>
-      <c r="H77" s="16"/>
+      <c r="H77" s="3"/>
       <c r="I77" s="3"/>
       <c r="J77" s="3"/>
       <c r="K77" s="3"/>
@@ -4219,7 +4205,7 @@
       <c r="E78" s="2"/>
       <c r="F78" s="2"/>
       <c r="G78" s="2"/>
-      <c r="H78" s="15"/>
+      <c r="H78" s="2"/>
       <c r="I78" s="2"/>
       <c r="J78" s="2"/>
       <c r="K78" s="2"/>
@@ -4250,7 +4236,7 @@
       <c r="E79" s="3"/>
       <c r="F79" s="3"/>
       <c r="G79" s="3"/>
-      <c r="H79" s="16"/>
+      <c r="H79" s="3"/>
       <c r="I79" s="3"/>
       <c r="J79" s="3"/>
       <c r="K79" s="3"/>
@@ -4281,7 +4267,7 @@
       <c r="E80" s="2"/>
       <c r="F80" s="2"/>
       <c r="G80" s="2"/>
-      <c r="H80" s="15"/>
+      <c r="H80" s="2"/>
       <c r="I80" s="2"/>
       <c r="J80" s="2"/>
       <c r="K80" s="2"/>
@@ -32848,27 +32834,27 @@
   <sheetData>
     <row r="1" spans="1:6" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="9" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="B1" s="9" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="9" t="s">
+        <v>258</v>
+      </c>
+      <c r="D1" s="9" t="s">
+        <v>259</v>
+      </c>
+      <c r="E1" s="9" t="s">
         <v>260</v>
       </c>
-      <c r="D1" s="9" t="s">
-        <v>261</v>
-      </c>
-      <c r="E1" s="9" t="s">
-        <v>262</v>
-      </c>
       <c r="F1" s="9" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="8" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="B2" s="8" t="s">
         <v>13</v>
@@ -32877,95 +32863,93 @@
         <v>13</v>
       </c>
       <c r="D2" s="8" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="E2" s="8" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="F2" s="14" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="8" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="B3" s="8" t="s">
         <v>47</v>
       </c>
       <c r="C3" s="8" t="s">
+        <v>265</v>
+      </c>
+      <c r="D3" s="8" t="s">
+        <v>266</v>
+      </c>
+      <c r="E3" s="8" t="s">
         <v>267</v>
       </c>
-      <c r="D3" s="8" t="s">
-        <v>268</v>
-      </c>
-      <c r="E3" s="8" t="s">
-        <v>269</v>
-      </c>
       <c r="F3" s="13" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="8" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="B4" s="8" t="s">
         <v>90</v>
       </c>
       <c r="C4" s="8" t="s">
+        <v>269</v>
+      </c>
+      <c r="D4" s="8" t="s">
+        <v>270</v>
+      </c>
+      <c r="E4" s="8" t="s">
         <v>271</v>
       </c>
-      <c r="D4" s="8" t="s">
-        <v>272</v>
-      </c>
-      <c r="E4" s="8" t="s">
-        <v>273</v>
-      </c>
       <c r="F4" s="13" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="8" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="B5" s="8" t="s">
         <v>107</v>
       </c>
       <c r="C5" s="8" t="s">
+        <v>273</v>
+      </c>
+      <c r="D5" s="8" t="s">
+        <v>274</v>
+      </c>
+      <c r="E5" s="8" t="s">
         <v>275</v>
       </c>
-      <c r="D5" s="8" t="s">
+      <c r="F5" s="13" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="8" t="s">
+        <v>380</v>
+      </c>
+      <c r="B6" s="8" t="s">
+        <v>339</v>
+      </c>
+      <c r="C6" s="8" t="s">
+        <v>339</v>
+      </c>
+      <c r="D6" s="8" t="s">
         <v>276</v>
       </c>
-      <c r="E5" s="8" t="s">
+      <c r="E6" s="8" t="s">
         <v>277</v>
       </c>
-      <c r="F5" s="13" t="s">
+      <c r="F6" s="13" t="s">
         <v>338</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="8" t="inlineStr">
-        <is>
-          <t>centro-multidisciplinar-de-angicos</t>
-        </is>
-      </c>
-      <c r="B6" s="8" t="s">
-        <v>341</v>
-      </c>
-      <c r="C6" s="8" t="s">
-        <v>341</v>
-      </c>
-      <c r="D6" s="8" t="s">
-        <v>278</v>
-      </c>
-      <c r="E6" s="8" t="s">
-        <v>279</v>
-      </c>
-      <c r="F6" s="13" t="s">
-        <v>340</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
@@ -32995,7 +32979,7 @@
   <sheetData>
     <row r="1" spans="1:3" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="9" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="B1" s="9" t="s">
         <v>4</v>
@@ -33006,7 +32990,7 @@
     </row>
     <row r="2" spans="1:3" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="8" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="B2" s="8" t="s">
         <v>13</v>
@@ -33017,7 +33001,7 @@
     </row>
     <row r="3" spans="1:3" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="8" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="B3" s="8" t="s">
         <v>13</v>
@@ -33028,7 +33012,7 @@
     </row>
     <row r="4" spans="1:3" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="8" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="B4" s="8" t="s">
         <v>47</v>
@@ -33039,7 +33023,7 @@
     </row>
     <row r="5" spans="1:3" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="8" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="B5" s="8" t="s">
         <v>47</v>
@@ -33050,7 +33034,7 @@
     </row>
     <row r="6" spans="1:3" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="8" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="B6" s="8" t="s">
         <v>47</v>
@@ -33061,7 +33045,7 @@
     </row>
     <row r="7" spans="1:3" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="8" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="B7" s="8" t="s">
         <v>90</v>
@@ -33072,7 +33056,7 @@
     </row>
     <row r="8" spans="1:3" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="8" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="B8" s="8" t="s">
         <v>90</v>
@@ -33083,7 +33067,7 @@
     </row>
     <row r="9" spans="1:3" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="8" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="B9" s="8" t="s">
         <v>107</v>
@@ -33094,7 +33078,7 @@
     </row>
     <row r="10" spans="1:3" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="8" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="B10" s="8" t="s">
         <v>107</v>
@@ -33105,7 +33089,7 @@
     </row>
     <row r="11" spans="1:3" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="8" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="B11" s="8" t="s">
         <v>107</v>
@@ -33116,7 +33100,7 @@
     </row>
     <row r="12" spans="1:3" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="8" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="B12" s="8" t="s">
         <v>107</v>
@@ -33127,7 +33111,7 @@
     </row>
     <row r="13" spans="1:3" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="8" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="B13" s="8" t="s">
         <v>107</v>
@@ -33138,7 +33122,7 @@
     </row>
     <row r="14" spans="1:3" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="8" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="B14" s="8" t="s">
         <v>107</v>
@@ -33149,7 +33133,7 @@
     </row>
     <row r="15" spans="1:3" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="8" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="B15" s="8" t="s">
         <v>107</v>
@@ -33160,46 +33144,46 @@
     </row>
     <row r="16" spans="1:3" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="8" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="C16" s="8" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="17" spans="1:3" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="8" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="18" spans="1:3" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="8" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="C18" s="8" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="19" spans="1:3" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="8" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="C19" s="8" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
   </sheetData>
@@ -33218,122 +33202,122 @@
   <sheetData>
     <row r="1" spans="1:2" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="11" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="B1" s="11" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="64.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="10" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="B2" s="10" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="64.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="10" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="64.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="10" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="64.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="10" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="64.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="10" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="64.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="10" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="64.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="10" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="64.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="10" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="64.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="10" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="B10" s="10" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="64.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="10" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="B11" s="10" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="64.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="10" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="B12" s="10" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="64.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="10" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="B13" s="10" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
     </row>
     <row r="14" spans="1:2" ht="64.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="10" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="B14" s="10" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
     </row>
     <row r="15" spans="1:2" ht="64.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="10" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="B15" s="10" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
     </row>
   </sheetData>

</xml_diff>